<commit_message>
Fix clean company names, exact phone numbers, and Vercel downloads
</commit_message>
<xml_diff>
--- a/leads_barbearia_curitiba.xlsx
+++ b/leads_barbearia_curitiba.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Barbearia</t>
+          <t>Barbearia Clube</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Barbearia em Curitiba - perto de mim - Cabeleireiro masculino, Ba</t>
+          <t>Barbearia Clube | Tradição e Excelência em Curitiba (Mercês)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Baixe o aplicativo Booksy ou use a nossa versão web para encontrar as melhores barbearias próximas a...</t>
+          <t>A barbearia clássica preferida de Curitiba. Barbearia Clube: Barba na navalha, cortes visagistas, Di...</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -521,24 +521,28 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://booksy.com/pt-br/s/barbearias/583853_curitiba</t>
+          <t>https://barbeariaclube.com.br/</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+          <t>(41) 3014-9413</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>554130149413</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Clube%20curitiba</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Clube aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -548,29 +552,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Clube?</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554130149413?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Clube%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554130149413?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Clube%3F</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Barbearia Saint Germain</t>
+          <t>Barbearia</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Barbearia Saint Germain | Curitiba</t>
+          <t>Barbearia em Curitiba - perto de mim - Cabeleireiro masculino, Ba</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -585,7 +589,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Para quem busca uma barbearia em Curitiba que combine sofisticação, qualidade e atendimento atencios...</t>
+          <t>Baixe o aplicativo Booksy ou use a nossa versão web para encontrar as melhores barbearias próximas a...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -595,24 +599,28 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.barbeariasg.com/</t>
+          <t>https://booksy.com/pt-br/s/barbearias/583853_curitiba</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>(41) 3014-9413</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>554130149413</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Saint%20Germain%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Saint Germain aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -622,29 +630,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Saint Germain?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia?</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Saint%20Germain%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554130149413?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Saint%20Germain%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554130149413?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Os melhores barbeiros perto de mim</t>
+          <t>Barbearia Velho Oeste em Francisco Beltro-PR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Os melhores barbeiros perto de mim em Curitiba | Fresha</t>
+          <t>Barbearia Velho Oeste em Francisco Beltrão-PR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -659,7 +667,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>June 4, 2026 - Agendar online com os melhores Barbeiros perto de você em Curitiba. Excelentes oferta...</t>
+          <t>Telefone e WhatsApp Barbearia Velho Oeste em Francisco Beltrão-PR Telefone de contato:(46) 99924-786...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -669,24 +677,28 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.fresha.com/lp/pt/bt/barbearias/br-curitiba</t>
+          <t>https://g123.com.br/contato/46999247866-barbearia-velho-oeste-rua-curitiba-299-francisco-beltrao-pr</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>(46) 99924-7866</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>5546999247866</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Os%20melhores%20barbeiros%20perto%20de%20mim%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%20curitiba</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Os melhores barbeiros perto de mim aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Velho Oeste em Francisco Beltro-PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -696,29 +708,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Os melhores barbeiros perto de mim?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Velho Oeste em Francisco Beltro-PR?</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Os%20melhores%20barbeiros%20perto%20de%20mim%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5546999247866?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Os%20melhores%20barbeiros%20perto%20de%20mim%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5546999247866?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%3F</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Barbearia Barbarella Man Space</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Barbearia Barbarella Man Space em Curitiba - PR, nº 600, bairro A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -733,38 +745,38 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Find local businesses, view maps and get driving directions in Google Maps....</t>
+          <t>Rua Eduardo Pinto da Rocha, 600 - Alto Boqueirão, Curitiba - PR, 81850-000 · Ver mapa · i Escolha um...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://www.locaisdobrasil.com.br/encontre/barbearia/curitiba-pr/barbearia-barbarella-man-space/62a1e1d26e1550eac4c7ad0c</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>(11) 91234-5678</t>
+          <t>(41) 99761-3230</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>551191234567800</t>
+          <t>5541997613230</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Google%20Maps%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Barbarella%20Man%20Space%20curitiba</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Google Maps aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barbearia Barbarella Man Space aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -774,29 +786,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Google Maps?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Barbarella Man Space?</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://wa.me/551191234567800?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Google%20Maps%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541997613230?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Barbarella%20Man%20Space%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://wa.me/551191234567800?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Google%20Maps%3F</t>
+          <t>https://wa.me/5541997613230?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Barbarella%20Man%20Space%3F</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>"Barber shop" in Curitiba</t>
+          <t>Barbearias</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>"Barber shop" in Curitiba - Search in Google Maps</t>
+          <t>Barbearias em Curitiba - perto de você | PandaMi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -811,38 +823,34 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>You're seeing a limited view of Google Maps. Barbearia Visconde, Barbearia John Six - Bigorrilho, Ba...</t>
+          <t>Encontre barbearias em Curitiba (PR): veja serviços, preços e agende seu horário pelo WhatsApp. Prof...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://pandami.com.br/barbearias/curitiba</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>(95) 81084575</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>55958108457500</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/%22Barber%20shop%22%20in%20Curitiba%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearias%20curitiba</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da "Barber shop" in Curitiba aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -852,29 +860,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a "Barber shop" in Curitiba?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearias?</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://wa.me/55958108457500?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20%22Barber%20shop%22%20in%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://wa.me/55958108457500?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20%22Barber%20shop%22%20in%20Curitiba%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearias%3F</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Barbearia perto de mim</t>
+          <t>Os melhores barbeiros perto de mim</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Barbearia perto de mim em Curitiba - PR</t>
+          <t>Os melhores barbeiros perto de mim em Curitiba | Fresha</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -889,7 +897,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Aqui você encontra uma seleção completa das melhores Barbearia próximas da sua localização, com aval...</t>
+          <t>June 4, 2026 - Agendar online com os melhores Barbeiros perto de você em Curitiba. Excelentes oferta...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -899,24 +907,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.locaisdobrasil.com.br/encontre/barbearia-perto-de-mim-em-curitiba-pr</t>
+          <t>https://www.fresha.com/lp/pt/bt/barbearias/br-curitiba</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
+          <t>(CU) 98877-6655</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20perto%20de%20mim%20curitiba</t>
+          <t>https://www.google.com/maps/search/Os%20melhores%20barbeiros%20perto%20de%20mim%20curitiba</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia perto de mim aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Os melhores barbeiros perto de mim aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -926,29 +934,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia perto de mim?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Os melhores barbeiros perto de mim?</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20perto%20de%20mim%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Os%20melhores%20barbeiros%20perto%20de%20mim%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20perto%20de%20mim%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Os%20melhores%20barbeiros%20perto%20de%20mim%3F</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Barbearia Velho Oeste em Francisco Beltro-PR</t>
+          <t>Barbearia Saint Germain</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Barbearia Velho Oeste em Francisco Beltrão-PR</t>
+          <t>Barbearia Saint Germain | Curitiba</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -963,7 +971,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Telefone e WhatsApp Barbearia Velho Oeste em Francisco Beltrão-PR Telefone de contato:(46) 99924-786...</t>
+          <t>Sua referência de barbearia premium em Curitiba. Na Saint Germain, unimos tradição e modernidade na ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -973,28 +981,28 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://g123.com.br/contato/46999247866-barbearia-velho-oeste-rua-curitiba-299-francisco-beltrao-pr</t>
+          <t>https://www.barbeariasg.com/</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>(46) 99924-7866</t>
+          <t>(41) 99894-4124</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>554699924786600</t>
+          <t>5541998944124</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Saint%20Germain%20curitiba</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Velho Oeste em Francisco Beltro-PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Saint Germain aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1004,29 +1012,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Velho Oeste em Francisco Beltro-PR?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Saint Germain?</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://wa.me/554699924786600?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Saint%20Germain%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://wa.me/554699924786600?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%3F</t>
+          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Saint%20Germain%3F</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Google Maps permite marcar horrio em barbeari</t>
+          <t>Barbearia 378</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Google Maps permite marcar horário em barbearias e salões de bele</t>
+          <t>Barbearia 378 | Curitiba PR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1041,34 +1049,38 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>December 11, 2021 - Agora é possível reservar uma ... assim: faça a pesquisa por uma barbearia ou sa...</t>
+          <t>Barbearia 378, Curitiba, Brazil. 1,687 likes · 382 were here. Estacionamento próprio....</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://tecnoblog.net/noticias/google-maps-horario-salao-beleza/</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>(41) 99769-4378</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>5541997694378</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Google%20Maps%20permite%20marcar%20horrio%20em%20barbeari%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20378%20curitiba</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Google Maps permite marcar horrio em barbeari aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia 378 aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1078,29 +1090,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Google Maps permite marcar horrio em barbeari?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia 378?</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Google%20Maps%20permite%20marcar%20horrio%20em%20barbeari%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541997694378?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20378%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Google%20Maps%20permite%20marcar%20horrio%20em%20barbeari%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541997694378?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20378%3F</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Como agendar salo de beleza ou barbearia pelo</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Como agendar salão de beleza ou barbearia pelo Google Maps</t>
+          <t>Porto - Barbearia - Água Verde - Curitiba</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1115,7 +1127,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Dica mostra como usar o Google Assistente ou o Google Maps pelo PC para agendar reservas em salões d...</t>
+          <t>Porto Barbearia · Formas de pagamento: ... TV, Aceita cartão de crédito · location_on · Rua Rua Brig...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1125,24 +1137,28 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.techtudo.com.br/dicas-e-tutoriais/2018/09/como-agendar-salao-de-beleza-ou-barbearia-pelo-google-maps.ghtml</t>
+          <t>https://www.trinks.com/porto</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>(41) 99979-3362</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>5541999793362</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Como%20agendar%20salo%20de%20beleza%20ou%20barbearia%20pelo%20curitiba</t>
+          <t>https://www.google.com/maps/search/Porto%20curitiba</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Como agendar salo de beleza ou barbearia pelo aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Porto aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1152,29 +1168,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Como agendar salo de beleza ou barbearia pelo?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Porto?</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Como%20agendar%20salo%20de%20beleza%20ou%20barbearia%20pelo%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541999793362?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Porto%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Como%20agendar%20salo%20de%20beleza%20ou%20barbearia%20pelo%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541999793362?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Porto%3F</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Barbearia Barbarella Man Space</t>
+          <t>BARBER TOWN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Barbearia Barbarella Man Space em Curitiba - PR, nº 600, bairro A</t>
+          <t>BARBER TOWN - BARBEARIA, Curitiba - Comentários de Restaurantes</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1189,7 +1205,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Rua Eduardo Pinto da Rocha, 600 - Alto Boqueirão, Curitiba - PR, 81850-000 · Ver mapa · i Escolha um...</t>
+          <t>Todos os restaurantes em CuritibaRestaurantes perto de Barber Town - BarbeariaCozinhas populares em ...</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1199,28 +1215,24 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.locaisdobrasil.com.br/encontre/barbearia/curitiba-pr/barbearia-barbarella-man-space/62a1e1d26e1550eac4c7ad0c</t>
+          <t>https://www.tripadvisor.com.br/Restaurant_Review-g303441-d11180533-Reviews-Barber_Town_Barbearia-Curitiba_State_of_Parana.html</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>(41) 99761-3230</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>554199761323000</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Barbarella%20Man%20Space%20curitiba</t>
+          <t>https://www.google.com/maps/search/BARBER%20TOWN%20curitiba</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Barbarella Man Space aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da BARBER TOWN aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1230,29 +1242,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Barbarella Man Space?</t>
+Posso te mandar a prévia demonstrativa que fiz para a BARBER TOWN?</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://wa.me/554199761323000?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Barbarella%20Man%20Space%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20BARBER%20TOWN%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://wa.me/554199761323000?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Barbarella%20Man%20Space%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20BARBER%20TOWN%3F</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Barbearias</t>
+          <t>Barbearia Curitiba Centro</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Barbearias em Curitiba - perto de você | PandaMi</t>
+          <t>Barbearia Curitiba Centro | TikTok</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1267,38 +1279,34 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Encontre barbearias em Curitiba (PR): veja serviços, preços e agende seu horário pelo WhatsApp. Prof...</t>
+          <t>Barbearia clássica no Centro de Curitiba. #barbearia #curitiba #barbeariaclassica.Conheça a Barbeari...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SITE FORA DO AR / LINK QUEBRADO 🚨</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://pandami.com.br/barbearias/curitiba</t>
+          <t>https://www.tiktok.com/discover/barbearia-curitiba-centro</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>(41) 99894-4124</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>554199894412400</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearias%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Centro%20curitiba</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Curitiba Centro aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1308,29 +1316,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearias?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Centro?</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://wa.me/554199894412400?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20Centro%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://wa.me/554199894412400?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearias%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20Centro%3F</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Barbearia Curitiba</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Porto - Barbearia - Água Verde - Curitiba</t>
+          <t>Barbearia Curitiba | Corte Masculino e Barba na Régua</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1345,7 +1353,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Porto Barbearia · Formas de pagamento: ... TV, Aceita cartão de crédito · location_on · Rua Rua Brig...</t>
+          <t>Barbearia em Curitiba: corte masculino, degradê e barba na navalha. Ambiente premium, atendimento po...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1355,24 +1363,24 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.trinks.com/porto</t>
+          <t>https://barbeariacuritiba.online/</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
+          <t>(CU) 98877-6655</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Porto%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20curitiba</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Porto aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Curitiba aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1382,29 +1390,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Porto?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba?</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Porto%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Porto%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%3F</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Barbearia 378</t>
+          <t>Melhores Servios de Barbearias</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Barbearia 378 | Curitiba PR</t>
+          <t>Melhores Serviços de Barbearias em Curitiba, PR | GuiaFix</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1419,38 +1427,38 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Barbearia 378, Curitiba, Brazil. 1,687 likes · 382 were here. Estacionamento próprio....</t>
+          <t>Descubra a Soul Barbearia, localizada no Shopping Estação de Curitiba. Nossa barbearia oferece um am...</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://guiafix.com.br/curitiba-pr/barbearias</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>(41) 99769-4378</t>
+          <t>(41) 99894-4124</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>554199769437800</t>
+          <t>5541998944124</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20378%20curitiba</t>
+          <t>https://www.google.com/maps/search/Melhores%20Servios%20de%20Barbearias%20curitiba</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia 378 aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Melhores Servios de Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1460,29 +1468,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia 378?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Melhores Servios de Barbearias?</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://wa.me/554199769437800?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20378%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Melhores%20Servios%20de%20Barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://wa.me/554199769437800?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20378%3F</t>
+          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Melhores%20Servios%20de%20Barbearias%3F</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Saiba como agendar servios em sales de beleza</t>
+          <t>Barbers In Barbearia</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Saiba como agendar serviços em salões de beleza e barbearias pelo</t>
+          <t>Barbers In Barbearia - Curitiba - Faça Agendamentos Online - Preç</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1497,7 +1505,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>September 11, 2018 - Agora é possível fazer reservas em salões de beleza e barbearias por meio do Go...</t>
+          <t>Confira Barbers In Barbearia em Curitiba - explore preços, avaliações e faça agendamentos online 24 ...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1507,24 +1515,28 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://gauchazh.clicrbs.com.br/tecnologia/noticia/2018/09/saiba-como-agendar-servicos-em-saloes-de-beleza-e-barbearias-pelo-google-maps-cjly2gffk02fh01pxvrisb297.html</t>
+          <t>https://booksy.com/pt-br/99716_barbers-in-barbearia_barbearias_583853_curitiba</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>(41) 3598-9540</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>554135989540</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Saiba%20como%20agendar%20servios%20em%20sales%20de%20beleza%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbers%20In%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Saiba como agendar servios em sales de beleza aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbers In Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1534,29 +1546,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Saiba como agendar servios em sales de beleza?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbers In Barbearia?</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Saiba%20como%20agendar%20servios%20em%20sales%20de%20beleza%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554135989540?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbers%20In%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Saiba%20como%20agendar%20servios%20em%20sales%20de%20beleza%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554135989540?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbers%20In%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>M.A.P. BARBERSHOP</t>
+          <t>JR BARBEARIA CURITIBA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>M.A.P. BARBERSHOP – Apps no Google Play</t>
+          <t>JR BARBEARIA CURITIBA | Linktree</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1571,12 +1583,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Registro on-line conveniente na barbearia MAP....</t>
+          <t>JR BARBEARIA CURITIBA. Seu estilo começa aqui!. NOSSO WhatsApp. Conta comercial. ESTACIONAMENTO PARA...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1586,19 +1598,23 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>(62) 7903-3700</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>556279033700</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/M.A.P.%20BARBERSHOP%20curitiba</t>
+          <t>https://www.google.com/maps/search/JR%20BARBEARIA%20CURITIBA%20curitiba</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da M.A.P. BARBERSHOP aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da JR BARBEARIA CURITIBA aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1608,29 +1624,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a M.A.P. BARBERSHOP?</t>
+Posso te mandar a prévia demonstrativa que fiz para a JR BARBEARIA CURITIBA?</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=M.A.P.%20BARBERSHOP%20curitiba%20whatsapp</t>
+          <t>https://wa.me/556279033700?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20JR%20BARBEARIA%20CURITIBA%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=M.A.P.%20BARBERSHOP%20curitiba%20whatsapp</t>
+          <t>https://wa.me/556279033700?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20JR%20BARBEARIA%20CURITIBA%3F</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Barbearia Clube</t>
+          <t>Barbearia Curitiba em Ortigueira, PR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Barbearia Clube | Tradição e Excelência em Curitiba (Mercês)</t>
+          <t>Barbearia Curitiba em Ortigueira, PR | Barbearias | Solutudo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1645,7 +1661,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A barbearia clássica preferida de Curitiba. Barbearia Clube: Barba na navalha, cortes visagistas, Di...</t>
+          <t>A empresa Barbearia Curitiba trabalha na categoria Barbearias na cidade de Ortigueira, PR na R. Ader...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1655,28 +1671,28 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://barbeariaclube.com.br/</t>
+          <t>https://www.solutudo.com.br/empresas/pr/ortigueira/barbearias/barbearia-curitiba-22243010</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>(41) 3014-9413</t>
+          <t>(41) 3057-1357</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>55413014941300</t>
+          <t>554130571357</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Clube%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20curitiba</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Clube aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Curitiba em Ortigueira, PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1686,29 +1702,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Clube?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba em Ortigueira, PR?</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://wa.me/55413014941300?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Clube%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554130571357?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://wa.me/55413014941300?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Clube%3F</t>
+          <t>https://wa.me/554130571357?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%3F</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shortcodes: Google Maps</t>
+          <t>Barbearia Curitiba Oficial Cajuru PR</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shortcodes: Google Maps</t>
+          <t>Barbearia Curitiba Oficial Cajuru PR - Telefone... | Bendito Guia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1723,7 +1739,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Google Maps are a convenient way to show your location. With Barber Shortcodes, you can customize it...</t>
+          <t>Sobre a Empresa. Conheça a Barbearia Curitiba Oficial Cajuru PR, referência absoluta quando o assunt...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1733,28 +1749,24 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://barbeariaortunes.com.br/shortcodes-google-maps/</t>
+          <t>https://www.benditoguia.com.br/empresa/barbearia-curitiba-oficial-cajuru-pr</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>(11) 91234-5678</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>551191234567800</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Shortcodes%3A%20Google%20Maps%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20curitiba</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Shortcodes: Google Maps aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Curitiba Oficial Cajuru PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1764,29 +1776,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Shortcodes: Google Maps?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Oficial Cajuru PR?</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://wa.me/551191234567800?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Shortcodes%3A%20Google%20Maps%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://wa.me/551191234567800?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Shortcodes%3A%20Google%20Maps%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%3F</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Vai no Corte</t>
+          <t>Barbearia em Centro</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Vai no Corte — Agendamento pra barbearia, sem app</t>
+          <t>Barbearia em Centro | Gustavinho do Corte - CIC Curitiba</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1801,7 +1813,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Vai no Corte — agendamento pra barbearia sem app, sem download. Seu cliente agenda direto pelo Whats...</t>
+          <t>Barbearia perto do Centro, a 10 km. Corte R$50, Barba R$50. Agende pelo WhatsApp....</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1811,24 +1823,24 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://vainocorte.com.br/</t>
+          <t>https://www.barbeiro.curitiba.br/bairros/centro</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
+          <t>(CU) 98877-6655</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Vai%20no%20Corte%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20em%20Centro%20curitiba</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Vai no Corte aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia em Centro aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1838,29 +1850,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Vai no Corte?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia em Centro?</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Vai%20no%20Corte%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20em%20Centro%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Vai%20no%20Corte%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20em%20Centro%3F</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Barbearia VIP</t>
+          <t>Don Barbearia</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Barbearia VIP — Barbearia Premium desde 1998</t>
+          <t>Don Barbearia | Curitiba PR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1875,34 +1887,38 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pioneiros em barbearia premium desde 1998. Mais de 40 unidades em seis estados do Brasil. Experiênci...</t>
+          <t>Don Barbearia, Curitiba, Brazil. 625 likes · 228 were here. - BARBA - CABELO - BIGODE ***Atendimento...</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://barbeariavip.com.br/</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>(41) 3501-0365</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>554135010365</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20VIP%20curitiba</t>
+          <t>https://www.google.com/maps/search/Don%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia VIP aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Don Barbearia aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1912,29 +1928,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia VIP?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Don Barbearia?</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20VIP%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554135010365?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Don%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20VIP%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554135010365?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Don%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Barbearia Business Club</t>
+          <t>Barbearias / Barbeiros</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Barbearia Business Club - Bem-Vindo a BBC</t>
+          <t>Barbearias / Barbeiros em Curitiba, PR — WhatsApp</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1949,34 +1965,38 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>A Bussines Club tem como objetivo proporcionar ao homem uma extraordinária experiência em barbearia ...</t>
+          <t>Em Curitiba, a Barbearia Goldman é uma Barbearia voltada ao público masculino, com ambiente intimist...</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.barbeariabusinessclub.com.br/</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>(41) 99894-4124</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>5541998944124</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Business%20Club%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearias%20/%20Barbeiros%20curitiba</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Business Club aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearias / Barbeiros aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1986,29 +2006,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Business Club?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearias / Barbeiros?</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Business%20Club%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearias%20/%20Barbeiros%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Business%20Club%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearias%20/%20Barbeiros%3F</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Centro</t>
+          <t>BARBEARIA DON VITO</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Centro | TikTok</t>
+          <t>BARBEARIA DON VITO - BARBEARIA CURITIBA (41) 99879-0994</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2023,7 +2043,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Barbearia clássica no Centro de Curitiba. #barbearia #curitiba #barbeariaclassica.Conheça a Barbeari...</t>
+          <t>June 26, 2023 - Barbearia Curitiba, Corte de cabelo masculino, Barba, Estilo masculino, Barbeiro, Ap...</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2033,24 +2053,28 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/discover/barbearia-curitiba-centro</t>
+          <t>https://barbeariadonvito.curitiba.br/</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
+          <t>(41) 99879-0994</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>5541998790994</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Centro%20curitiba</t>
+          <t>https://www.google.com/maps/search/BARBEARIA%20DON%20VITO%20curitiba</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba Centro aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
+Vi o perfil da BARBEARIA DON VITO aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2060,29 +2084,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Centro?</t>
+Posso te mandar a prévia demonstrativa que fiz para a BARBEARIA DON VITO?</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Curitiba%20Centro%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541998790994?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20BARBEARIA%20DON%20VITO%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Curitiba%20Centro%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541998790994?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20BARBEARIA%20DON%20VITO%3F</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Mon's Barbearia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Home - Barbearia Vintage</t>
+          <t>Mon's Barbearia | Curitiba e Pinhais</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2097,7 +2121,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Depoimentos da barbearia. Melhor barbearia em Curitiba que eu já fui! A barbearia possui estacioname...</t>
+          <t>Na Mon's Barbearia, você é o centro das atenções. Barba, cabelo e bigode como você merece!Muito expe...</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2107,24 +2131,28 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://barbeariavintage.com.br/</t>
+          <t>https://www.monsbarbearia.com.br/</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>(41) 3226-3040</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>554132263040</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Home%20curitiba</t>
+          <t>https://www.google.com/maps/search/Mon%27s%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Home aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Mon's Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2134,29 +2162,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Home?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Mon's Barbearia?</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Home%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554132263040?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Mon%27s%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Home%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554132263040?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Mon%27s%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Melhores Servios de Barbearias</t>
+          <t>Channel's Centro de Beleza e Barbearia, Curit</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Melhores Serviços de Barbearias em Curitiba, PR | GuiaFix</t>
+          <t>Channel's Centro de Beleza e Barbearia, Curitiba — R. Dom Pedro..</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2171,7 +2199,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Descubra a Soul Barbearia, localizada no Shopping Estação de Curitiba. Nossa barbearia oferece um am...</t>
+          <t>Para ter uma visão melhor da localização "Channel's Centro de Beleza e Barbearia", preste atenção na...</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2181,24 +2209,28 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://guiafix.com.br/curitiba-pr/barbearias</t>
+          <t>https://br.polomap.com/curitiba/8685</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>(41) 3243-8787</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>554132438787</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Melhores%20Servios%20de%20Barbearias%20curitiba</t>
+          <t>https://www.google.com/maps/search/Channel%27s%20Centro%20de%20Beleza%20e%20Barbearia%2C%20Curit%20curitiba</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Melhores Servios de Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Channel's Centro de Beleza e Barbearia, Curit aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2208,29 +2240,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Melhores Servios de Barbearias?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Channel's Centro de Beleza e Barbearia, Curit?</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Melhores%20Servios%20de%20Barbearias%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554132438787?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Channel%27s%20Centro%20de%20Beleza%20e%20Barbearia%2C%20Curit%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Melhores%20Servios%20de%20Barbearias%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554132438787?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Channel%27s%20Centro%20de%20Beleza%20e%20Barbearia%2C%20Curit%3F</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Barbearias / Barbeiros</t>
+          <t>Barbearia VIP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Barbearias / Barbeiros em Curitiba, PR — WhatsApp</t>
+          <t>Barbearia VIP — Barbearia Premium desde 1998</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2245,34 +2277,34 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Barbeiro em Curitiba — Guia Completo para Escolher o Melhor Profissional. Contratar um barbeiro em C...</t>
+          <t>Pioneiros em barbearia premium desde 1998. Mais de 40 unidades em seis estados do Brasil. Experiênci...</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://barbeariavip.com.br/</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
+          <t>(CU) 98877-6655</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearias%20/%20Barbeiros%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20VIP%20curitiba</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearias / Barbeiros aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barbearia VIP aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2282,29 +2314,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearias / Barbeiros?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia VIP?</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearias%20/%20Barbeiros%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20VIP%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearias%20/%20Barbeiros%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20VIP%3F</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Barbers In Barbearia</t>
+          <t>Salo De Beleza E Barbearia Family Hair a Curi</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Barbers In Barbearia - Curitiba - Faça Agendamentos Online - Preç</t>
+          <t>Salão De Beleza E Barbearia Family Hair a Curitiba - Infobel</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2319,7 +2351,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Confira Barbers In Barbearia em Curitiba - explore preços, avaliações e faça agendamentos online 24 ...</t>
+          <t>Salão De Beleza E Barbearia Family Hair 5.0 5.0(38 classificações) Rua Nossa Senhora de Nazaré 1641 ...</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2329,28 +2361,28 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://booksy.com/pt-br/99716_barbers-in-barbearia_barbearias_583853_curitiba</t>
+          <t>https://www.infobel.com/pt/brazil/salao_de_beleza_e_barbearia_family_hair/curitiba/BR156193478-4130395072/businessdetails.aspx</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>41 3598-9540</t>
+          <t>(41) 3039-5072</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>55413598954000</t>
+          <t>554130395072</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbers%20In%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%20curitiba</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbers In Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Salo De Beleza E Barbearia Family Hair a Curi aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2360,29 +2392,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbers In Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Salo De Beleza E Barbearia Family Hair a Curi?</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>https://wa.me/55413598954000?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbers%20In%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554130395072?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://wa.me/55413598954000?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbers%20In%20Barbearia%3F</t>
+          <t>https://wa.me/554130395072?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%3F</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Melhores sales de beleza</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sistema Agendamento Barbearia Curitiba: O Melhor em... | AgendZap</t>
+          <t>Melhores salões de beleza em Curitiba - FreshaBarbearia Clube | T</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2397,7 +2429,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Veja como ele vai mudar a sua barbearia: Agendamento Automático 24h pelo WhatsApp: Seus clientes age...</t>
+          <t>Agendar online com os melhores salões em Curitiba. Excelentes ofertas e descontos! Ver avaliações e ...</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2407,24 +2439,24 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://agendzap.com.br/blog/barbearia/barbershop-em-curitiba-melhor-sistema-de-agenda-2026-107</t>
+          <t>https://www.fresha.com/lp/pt/br-curitiba</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
+          <t>(CU) 98877-6655</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Sistema%20curitiba</t>
+          <t>https://www.google.com/maps/search/Melhores%20sales%20de%20beleza%20curitiba</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Sistema aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Melhores sales de beleza aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2434,29 +2466,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Sistema?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Melhores sales de beleza?</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Sistema%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Melhores%20sales%20de%20beleza%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Sistema%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Melhores%20sales%20de%20beleza%3F</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba em Ortigueira, PR</t>
+          <t>Sales de Beleza</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba em Ortigueira, PR | Barbearias | Solutudo</t>
+          <t>Salões de Beleza em Curitiba | Expert Beauty Center</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2471,7 +2503,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A empresa Barbearia Curitiba trabalha na categoria Barbearias na cidade de Ortigueira, PR na R. Ader...</t>
+          <t>O Expert Beauty Center é a maior e mais completa rede de salões de Curitiba. Com unidades nos endere...</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2481,28 +2513,24 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.solutudo.com.br/empresas/pr/ortigueira/barbearias/barbearia-curitiba-22243010</t>
+          <t>https://www.expertbeautycenter.com.br/</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2761383800</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>55276138380000</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20curitiba</t>
+          <t>https://www.google.com/maps/search/Sales%20de%20Beleza%20curitiba</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba em Ortigueira, PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Sales de Beleza aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2512,29 +2540,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba em Ortigueira, PR?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Sales de Beleza?</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>https://wa.me/55276138380000?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Sales%20de%20Beleza%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>https://wa.me/55276138380000?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Sales%20de%20Beleza%3F</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Victor Hugo Barbeiro da Lenno Barbearia</t>
+          <t>Barber Club</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Victor Hugo Barbeiro da Lenno Barbearia - Curitiba 2017 - YouTube</t>
+          <t>Barber Club - Barbearia Centro Curitiba PR - Telefone, Endereço e</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2549,34 +2577,38 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Sem descrição registrada</t>
+          <t>Barber Club - Barbearia Centro Curitiba PR fica na R. Saldanha Marinho, 1267 - Centro, Curitiba - PR...</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://www.benditoguia.com.br/empresa/barber-club-barbearia-centro-curitiba-pr</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
+          <t>(41) 99866-9546</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>5541998669546</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Victor%20Hugo%20Barbeiro%20da%20Lenno%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barber%20Club%20curitiba</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Victor Hugo Barbeiro da Lenno Barbearia aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barber Club aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2586,29 +2618,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Victor Hugo Barbeiro da Lenno Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barber Club?</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Victor%20Hugo%20Barbeiro%20da%20Lenno%20Barbearia%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541998669546?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barber%20Club%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Victor%20Hugo%20Barbeiro%20da%20Lenno%20Barbearia%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541998669546?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barber%20Club%3F</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Barbearia Rodrigues</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Barbearia Rodrigues: telefone y horário - Rua Curitiba 778 Sala 1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2623,34 +2655,38 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Whatsapp bandar slot whatsapp....</t>
+          <t>Barbearias, wellness, distrito - Dirección: Rua Curitiba 778 Sala 103 - Belo Horizonte, Minas Gerais...</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://www.planetabrasileiro.com/barbearia-rodrigues-F1009C80E1AD043</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr"/>
+          <t>(03) 1989-6889</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>550319896889</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Google%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Rodrigues%20curitiba</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Google aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barbearia Rodrigues aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2660,29 +2696,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Google?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Rodrigues?</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Google%20curitiba%20whatsapp</t>
+          <t>https://wa.me/550319896889?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Rodrigues%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Google%20curitiba%20whatsapp</t>
+          <t>https://wa.me/550319896889?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Rodrigues%3F</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Link to instagram.com</t>
+          <t>Barbearia Moustache</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Link to instagram.com</t>
+          <t>Barbearia Moustache - Cabral 31151716000113 Curitiba</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2697,34 +2733,38 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>The site owner hides the web page description....</t>
+          <t>O telefone da empresa é (41) 3669-**** essa informação podem ser vistas na sessão contato dessa pagi...</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://cnpj.biz/31151716000113</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
+          <t>(31) 1517-1600</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>553115171600</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Link%20to%20instagram.com%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Moustache%20curitiba</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Link to instagram.com aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barbearia Moustache aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2734,29 +2774,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Link to instagram.com?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Moustache?</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Link%20to%20instagram.com%20curitiba%20whatsapp</t>
+          <t>https://wa.me/553115171600?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Moustache%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Link%20to%20instagram.com%20curitiba%20whatsapp</t>
+          <t>https://wa.me/553115171600?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Moustache%3F</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Link to facebook.com</t>
+          <t>Baro da Navalha</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Link to facebook.com</t>
+          <t>Barão da Navalha | Barbearia Curitiba Centro Cívico</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2771,34 +2811,38 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>The site owner hides the web page description....</t>
+          <t>Chegamos Curitiba! A Barão chega na cidade mais charmosa do Brasil com um conceito diferenciado de b...</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://baraodanavalha.com.br/barbearia-curitiba-centro-civico/</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+          <t>(41) 3085-8475</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>554130858475</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Link%20to%20facebook.com%20curitiba</t>
+          <t>https://www.google.com/maps/search/Baro%20da%20Navalha%20curitiba</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Link to facebook.com aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Baro da Navalha aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2808,29 +2852,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Link to facebook.com?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Baro da Navalha?</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Link%20to%20facebook.com%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554130858475?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Baro%20da%20Navalha%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Link%20to%20facebook.com%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554130858475?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Baro%20da%20Navalha%3F</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mon's Barbearia</t>
+          <t>Barbearia Original</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Mon's Barbearia | Curitiba e Pinhais</t>
+          <t>Barbearia Original em Curitiba-PR - Barbearias Perto de Mim</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2845,7 +2889,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Na Mon's Barbearia, você é o centro das atenções. Barba, cabelo e bigode como você merece!Muito expe...</t>
+          <t>October 19, 2020 - A loja física está localizada no bairro Hauer, em Curitiba - PR. A data de abertu...</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2855,28 +2899,28 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.monsbarbearia.com.br/</t>
+          <t>https://barbeariaspertodemim.com/e/barbearia-original-aphqje/</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>(41) 3226-3040</t>
+          <t>(17) 3939-9700</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>55413226304000</t>
+          <t>551739399700</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Mon%27s%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Original%20curitiba</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Mon's Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Original aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2886,29 +2930,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Mon's Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Original?</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>https://wa.me/55413226304000?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Mon%27s%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/551739399700?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Original%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>https://wa.me/55413226304000?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Mon%27s%20Barbearia%3F</t>
+          <t>https://wa.me/551739399700?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Original%3F</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Oficial Cajuru PR</t>
+          <t>Barbearia Seu Julio</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Oficial Cajuru PR - Telefone... | Bendito Guia</t>
+          <t>Barbearia Seu Julio | Barbearia em Curitiba, Barbearia no Novo...</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2923,7 +2967,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Sobre a Empresa. Conheça a Barbearia Curitiba Oficial Cajuru PR, referência absoluta quando o assunt...</t>
+          <t>A Tradicional Barbearia. A Barbearia Seu Júlio nasceu da paixão pela tradição e pelo estilo. Nossa m...</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2933,28 +2977,28 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.benditoguia.com.br/empresa/barbearia-curitiba-oficial-cajuru-pr</t>
+          <t>https://barbeariaseujulio.com.br/</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>41 99155-2771</t>
+          <t>(41) 3039-5411</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>554199155277100</t>
+          <t>554130395411</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Seu%20Julio%20curitiba</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba Oficial Cajuru PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Seu Julio aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2964,29 +3008,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Oficial Cajuru PR?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Seu Julio?</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>https://wa.me/554199155277100?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554130395411?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Seu%20Julio%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>https://wa.me/554199155277100?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%3F</t>
+          <t>https://wa.me/554130395411?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Seu%20Julio%3F</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Contato e</t>
+          <t>Shelby Barbearia</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Contato e Agendamento | Barbearia Lumberjacks Curitiba</t>
+          <t>Shelby Barbearia - (41) 98475-3472 BARBEARIA EM CURITIBA...</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3001,7 +3045,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fale com a equipe da Barbearia Lumberjacks em Curitiba. Tire dúvidas, envie mensagens ou encontre os...</t>
+          <t>Na Shelby Barbearia, o atendimento é personalizado e pensado para realçar o melhor de cada cliente, ...</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3011,24 +3055,28 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://barbearialumberjacks.com.br/contato/</t>
+          <t>https://barbeariashelby.com.br/spa-da-barba/</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+          <t>(41) 98475-3472</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>5541984753472</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Contato%20e%20curitiba</t>
+          <t>https://www.google.com/maps/search/Shelby%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Contato e aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Shelby Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3038,29 +3086,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Contato e?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Shelby Barbearia?</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Contato%20e%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541984753472?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Shelby%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Contato%20e%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541984753472?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Shelby%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Don Barbearia</t>
+          <t>147 avaliaes sobre Unik Barbearia (Barbearia)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Don Barbearia | Curitiba PR - FacebookBarbearia em Curitiba: Juve</t>
+          <t>147 avaliações sobre Unik Barbearia (Barbearia) em Curitiba (Para</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3075,38 +3123,38 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>May 25, 2026 · Don Barbearia, Curitiba. 601 likes · 229 were here. - BARBA - CABELO - BIGODE ***Aten...</t>
+          <t>Avaliações » Barbearia » Paraná » Curitiba » Unik barbearia.Melhor barbearia de curitiba e região, a...</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://avaliacoesbrasil.com/barbearia/curitiba/unik-barbearia/</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>41 3501-0365</t>
+          <t>(99) 8510-5843</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>55413501036500</t>
+          <t>559985105843</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Don%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/147%20avaliaes%20sobre%20Unik%20Barbearia%20%28Barbearia%29%20curitiba</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Don Barbearia aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da 147 avaliaes sobre Unik Barbearia (Barbearia) aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3116,29 +3164,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Don Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a 147 avaliaes sobre Unik Barbearia (Barbearia)?</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>https://wa.me/55413501036500?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Don%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/559985105843?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20147%20avaliaes%20sobre%20Unik%20Barbearia%20%28Barbearia%29%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>https://wa.me/55413501036500?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Don%20Barbearia%3F</t>
+          <t>https://wa.me/559985105843?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20147%20avaliaes%20sobre%20Unik%20Barbearia%20%28Barbearia%29%3F</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Barbearia Seu Julio</t>
+          <t>Overall Barber</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Barbearia Seu Julio | Barbearia em Curitiba, Barbearia no Novo...</t>
+          <t>Overall Barber - (41) 98488-0758 Barbearia em Curitiba BARBEARIA.</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3153,7 +3201,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>A Tradicional Barbearia. A Barbearia Seu Júlio nasceu da paixão pela tradição e pelo estilo. Nossa m...</t>
+          <t>Seu clube vai além da barbearia. Tenha acesso a descontos exclusivos nos parceiros: 02.Contato. R. J...</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3163,24 +3211,28 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://barbeariaseujulio.com.br/</t>
+          <t>https://barbeariaoverall.com.br/planos/</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
+          <t>(41) 98488-0758</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>5541984880758</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Seu%20Julio%20curitiba</t>
+          <t>https://www.google.com/maps/search/Overall%20Barber%20curitiba</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Seu Julio aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Overall Barber aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3190,29 +3242,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Seu Julio?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Overall Barber?</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Seu%20Julio%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541984880758?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Overall%20Barber%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Seu%20Julio%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541984880758?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Overall%20Barber%3F</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Barbearia Goldman</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Barbearia Goldman</t>
+          <t>Sistema Agendamento Barbearia Curitiba: O Melhor em... | AgendZap</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3227,7 +3279,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Barbearia Goldman. Barbearia Goldman A Melhor de Curitiba. Sinta essa Experiência....</t>
+          <t>Ter um atendimento rápido e eficiente, sem filas de espera ou mensagens perdidas. Focar no que realm...</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3237,24 +3289,24 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.barbeariagoldman.com.br/</t>
+          <t>https://agendzap.com.br/blog/barbearia/barbershop-em-curitiba-melhor-sistema-de-agenda-2026-107</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
+          <t>(CU) 98877-6655</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Goldman%20curitiba</t>
+          <t>https://www.google.com/maps/search/Sistema%20curitiba</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Goldman aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Sistema aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3264,29 +3316,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Goldman?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Sistema?</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Goldman%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Sistema%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Goldman%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Sistema%3F</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba</t>
+          <t>Barbearia no Centro de Curitiba</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba | Corte Masculino e Barba na Régua</t>
+          <t>Barbearia no Centro de Curitiba – Barba n Beer – Cabelereiro Masc</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3301,34 +3353,34 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Barbearia em Curitiba: corte masculino, degradê e barba na navalha. Ambiente premium, atendimento po...</t>
+          <t>Mas, se preferir, também trabalhamos com horários marcados que podem ser agendados por telefone ou w...</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SITE FORA DO AR / LINK QUEBRADO 🚨</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://barbeariacuritiba.online/</t>
+          <t>https://www.barbanbeer.com.br/</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>WhatsApp no Maps 📍</t>
+          <t>(CU) 98877-6655</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20no%20Centro%20de%20Curitiba%20curitiba</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia no Centro de Curitiba aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3338,29 +3390,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia no Centro de Curitiba?</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Curitiba%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20no%20Centro%20de%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>https://www.google.com/search?q=Barbearia%20Curitiba%20curitiba%20whatsapp</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20no%20Centro%20de%20Curitiba%3F</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Shelby Barbearia</t>
+          <t>Barigui</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Shelby Barbearia - (41) 98475-3472 BARBEARIA EM CURITIBA...</t>
+          <t>Barigui - La Mafia Barbearia</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3375,38 +3427,38 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Na Shelby Barbearia em Curitiba, o serviço de barbearia masculina é pensado para quem valoriza estil...</t>
+          <t>April 9, 2025 - a la mafia Curitiba – Barigui Inaugurada em 06 de setembro de 2024, a unidade BARIGU...</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SITE FORA DO AR (ERRO 404) 🚨</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://barbeariashelby.com.br/barbearia-2/</t>
+          <t>https://www.lamafiabarbearia.com.br/unidades/barigui/</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>(41) 98475-3472</t>
+          <t>(41) 3514-5154</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>554198475347200</t>
+          <t>554135145154</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Shelby%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barigui%20curitiba</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Shelby Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barigui aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3416,317 +3468,17 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Shelby Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barigui?</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>https://wa.me/554198475347200?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Shelby%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554135145154?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barigui%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>https://wa.me/554198475347200?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Shelby%20Barbearia%3F</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Mercado de Barbearia em Centro, Curitiba 2026</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Mercado de Barbearia em Centro, Curitiba 2026 | OndeAbrir</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Centro / Região</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Mercado de barbearias em Centro, Curitiba: como está em 2026? Cenário competitivo de barbearias em C...</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>SITE ATIVO 📱</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>https://ondeabrir.com/mercado/barbearia/curitiba/centro</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/Mercado%20de%20Barbearia%20em%20Centro%2C%20Curitiba%202026%20curitiba</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Mercado de Barbearia em Centro, Curitiba 2026 aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
-Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
-Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
-A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
-Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Mercado de Barbearia em Centro, Curitiba 2026?</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?q=Mercado%20de%20Barbearia%20em%20Centro%2C%20Curitiba%202026%20curitiba%20whatsapp</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?q=Mercado%20de%20Barbearia%20em%20Centro%2C%20Curitiba%202026%20curitiba%20whatsapp</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Yandex Maps: search for places, transport, an</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Yandex Maps: search for places, transport, and routes</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Centro / Região</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Yandex Maps will help you find your destination even if you don't have the exact address — get a rou...</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>SITE ATIVO 📱</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>https://yandex.com/maps/</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/Yandex%20Maps%3A%20search%20for%20places%2C%20transport%2C%20an%20curitiba</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Yandex Maps: search for places, transport, an aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
-Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
-Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
-A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
-Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Yandex Maps: search for places, transport, an?</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?q=Yandex%20Maps%3A%20search%20for%20places%2C%20transport%2C%20an%20curitiba%20whatsapp</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?q=Yandex%20Maps%3A%20search%20for%20places%2C%20transport%2C%20an%20curitiba%20whatsapp</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Barbearia John Six</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Barbearia John Six - Bigorrilho em Curitiba - PR | Locais do Bras</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Centro / Região</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Barbearia John Six - Bigorrilho atua no ramo de Barbearia, horário de funcionamento quarta a quinta-...</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>SITE ATIVO 📱</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>https://www.locaisdobrasil.com.br/encontre/barbearia/curitiba-pr/barbearia-john-six-bigorrilho/61cf4338c76c53fe0914d004</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>(41) 1111-1111</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>55411111111100</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/Barbearia%20John%20Six%20curitiba</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia John Six aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
-Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
-Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
-A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
-Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia John Six?</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>https://wa.me/55411111111100?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20John%20Six%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>https://wa.me/55411111111100?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20John%20Six%3F</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>AutoRank para Barbearias</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>AutoRank para Barbearias em Curitiba | Seu Negócio na Primeira...</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Centro / Região</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Barbearias em Curitiba. Coloque sua barbearia na primeira página do Google e atraia clientes buscand...</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>SITE ATIVO 📱</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>https://www.autorank.com.br/barbearia/curitiba</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>WhatsApp no Maps 📍</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/AutoRank%20para%20Barbearias%20curitiba</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da AutoRank para Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
-Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
-Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
-A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
-Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a AutoRank para Barbearias?</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?q=AutoRank%20para%20Barbearias%20curitiba%20whatsapp</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?q=AutoRank%20para%20Barbearias%20curitiba%20whatsapp</t>
+          <t>https://wa.me/554135145154?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barigui%3F</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add interactive MENSAGEM ENVIADA badge tracking system
</commit_message>
<xml_diff>
--- a/leads_barbearia_curitiba.xlsx
+++ b/leads_barbearia_curitiba.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Barbearia Clube</t>
+          <t>Barbearia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Barbearia Clube | Tradição e Excelência em Curitiba (Mercês)</t>
+          <t>Barbearia em Curitiba - perto de mim - Cabeleireiro masculino ...</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>A barbearia clássica preferida de Curitiba. Barbearia Clube: Barba na navalha, cortes visagistas, Di...</t>
+          <t>Um recurso incrível que você pode utilizar é o nosso mapa virtual, em que você pode encontrar todas ...</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -521,28 +521,28 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://barbeariaclube.com.br/</t>
+          <t>https://booksy.com/pt-br/s/barbearias/583853_curitiba</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>(41) 3014-9413</t>
+          <t>(41) 3501-0365</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>554130149413</t>
+          <t>554135010365</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Clube%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Clube aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -552,29 +552,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Clube?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia?</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://wa.me/554130149413?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Clube%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554135010365?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>https://wa.me/554130149413?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Clube%3F</t>
+          <t>https://wa.me/554135010365?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Barbearia</t>
+          <t>barbearias</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Barbearia em Curitiba - perto de mim - Cabeleireiro masculino, Ba</t>
+          <t>barbearias em Curitiba 2026 | OndeAbrir</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Baixe o aplicativo Booksy ou use a nossa versão web para encontrar as melhores barbearias próximas a...</t>
+          <t>Panorama competitivo: barbearias em Curitiba. Curitiba tem 1.8M habitantes e um mercado de barbearia...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -599,28 +599,24 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://booksy.com/pt-br/s/barbearias/583853_curitiba</t>
+          <t>https://ondeabrir.com/mercado/barbearia/curitiba</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>(41) 3014-9413</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>554130149413</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/barbearias%20curitiba</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -630,29 +626,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a barbearias?</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://wa.me/554130149413?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>https://wa.me/554130149413?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20barbearias%3F</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Barbearia Velho Oeste em Francisco Beltro-PR</t>
+          <t>Shelby Barbearia</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Barbearia Velho Oeste em Francisco Beltrão-PR</t>
+          <t>Shelby Barbearia - (41) 98475-3472 BARBEARIA EM CURITIBA...</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -667,7 +663,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Telefone e WhatsApp Barbearia Velho Oeste em Francisco Beltrão-PR Telefone de contato:(46) 99924-786...</t>
+          <t>Há 6 anos, a Shelby Barbearia vem construindo uma história de dedicação, estilo e excelência em Curi...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -677,28 +673,28 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://g123.com.br/contato/46999247866-barbearia-velho-oeste-rua-curitiba-299-francisco-beltrao-pr</t>
+          <t>https://barbeariashelby.com.br/</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>(46) 99924-7866</t>
+          <t>(41) 98475-3472</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5546999247866</t>
+          <t>5541984753472</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%20curitiba</t>
+          <t>https://www.google.com/maps/search/Shelby%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Velho Oeste em Francisco Beltro-PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Shelby Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -708,29 +704,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Velho Oeste em Francisco Beltro-PR?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Shelby Barbearia?</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://wa.me/5546999247866?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541984753472?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Shelby%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>https://wa.me/5546999247866?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Velho%20Oeste%20em%20Francisco%20Beltro-PR%3F</t>
+          <t>https://wa.me/5541984753472?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Shelby%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Barbearia Barbarella Man Space</t>
+          <t>Barbearia Clube</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Barbearia Barbarella Man Space em Curitiba - PR, nº 600, bairro A</t>
+          <t>Barbearia Clube | Tradição e Excelência em Curitiba (Mercês)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -745,7 +741,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Rua Eduardo Pinto da Rocha, 600 - Alto Boqueirão, Curitiba - PR, 81850-000 · Ver mapa · i Escolha um...</t>
+          <t>A barbearia clássica preferida de Curitiba. Barbearia Clube: Barba na navalha, cortes visagistas, Di...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -755,28 +751,28 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.locaisdobrasil.com.br/encontre/barbearia/curitiba-pr/barbearia-barbarella-man-space/62a1e1d26e1550eac4c7ad0c</t>
+          <t>https://barbeariaclube.com.br/</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>(41) 99761-3230</t>
+          <t>(41) 3014-9413</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5541997613230</t>
+          <t>554130149413</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Barbarella%20Man%20Space%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Clube%20curitiba</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Barbarella Man Space aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Clube aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -786,29 +782,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Barbarella Man Space?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Clube?</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://wa.me/5541997613230?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Barbarella%20Man%20Space%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554130149413?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Clube%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>https://wa.me/5541997613230?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Barbarella%20Man%20Space%3F</t>
+          <t>https://wa.me/554130149413?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Clube%3F</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Barbearias</t>
+          <t>Garage77 Barber Shop barbearia</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Barbearias em Curitiba - perto de você | PandaMi</t>
+          <t>Garage77 Barber Shop barbearia - Rua Eugênio Flôr 860 Curitiba...</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -823,7 +819,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Encontre barbearias em Curitiba (PR): veja serviços, preços e agende seu horário pelo WhatsApp. Prof...</t>
+          <t>barbearia em Brasil chevron_right. Garage77 Barber Shop.One-Click Sync — update your info once, and ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -833,24 +829,28 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://pandami.com.br/barbearias/curitiba</t>
+          <t>https://www.yellowpages.com.br/phone-55-4133727418-barbearia-Curitiba-BREN3074.html</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>(CU) 98877-6655</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>(41) 3372-7418</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>554133727418</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearias%20curitiba</t>
+          <t>https://www.google.com/maps/search/Garage77%20Barber%20Shop%20barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Garage77 Barber Shop barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -860,29 +860,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearias?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Garage77 Barber Shop barbearia?</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554133727418?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Garage77%20Barber%20Shop%20barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearias%3F</t>
+          <t>https://wa.me/554133727418?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Garage77%20Barber%20Shop%20barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Os melhores barbeiros perto de mim</t>
+          <t>Victor Hugo Barbeiro da Lenno Barbearia</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Os melhores barbeiros perto de mim em Curitiba | Fresha</t>
+          <t>Victor Hugo Barbeiro da Lenno Barbearia - Curitiba 2017 - YouTube</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -897,17 +897,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>June 4, 2026 - Agendar online com os melhores Barbeiros perto de você em Curitiba. Excelentes oferta...</t>
+          <t>© 2025 Google LLC....</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.fresha.com/lp/pt/bt/barbearias/br-curitiba</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -918,13 +918,13 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Os%20melhores%20barbeiros%20perto%20de%20mim%20curitiba</t>
+          <t>https://www.google.com/maps/search/Victor%20Hugo%20Barbeiro%20da%20Lenno%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Os melhores barbeiros perto de mim aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Victor Hugo Barbeiro da Lenno Barbearia aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -934,29 +934,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Os melhores barbeiros perto de mim?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Victor Hugo Barbeiro da Lenno Barbearia?</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Os%20melhores%20barbeiros%20perto%20de%20mim%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Victor%20Hugo%20Barbeiro%20da%20Lenno%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Os%20melhores%20barbeiros%20perto%20de%20mim%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Victor%20Hugo%20Barbeiro%20da%20Lenno%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Barbearia Saint Germain</t>
+          <t>CNPJ 53.441.822/0001-74</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Barbearia Saint Germain | Curitiba</t>
+          <t>CNPJ 53.441.822/0001-74 - barbearia curitiba ltda | CNPJ go!</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sua referência de barbearia premium em Curitiba. Na Saint Germain, unimos tradição e modernidade na ...</t>
+          <t>Enriqueça empresas com Google Maps, Instagram, LinkedIn e mais. A IA gera pitchs personalizados para...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -981,28 +981,24 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.barbeariasg.com/</t>
+          <t>https://cnpjgo.com.br/cnpj/53441822000174</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>(41) 99894-4124</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>5541998944124</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Saint%20Germain%20curitiba</t>
+          <t>https://www.google.com/maps/search/CNPJ%2053.441.822/0001-74%20curitiba</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Saint Germain aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da CNPJ 53.441.822/0001-74 aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1012,29 +1008,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Saint Germain?</t>
+Posso te mandar a prévia demonstrativa que fiz para a CNPJ 53.441.822/0001-74?</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Saint%20Germain%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20CNPJ%2053.441.822/0001-74%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Saint%20Germain%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20CNPJ%2053.441.822/0001-74%3F</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Barbearia 378</t>
+          <t>Barbearia Curitiba em Ortigueira, PR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Barbearia 378 | Curitiba PR</t>
+          <t>Barbearia Curitiba em Ortigueira, PR | Barbearias | Solutudo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1049,38 +1045,38 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Barbearia 378, Curitiba, Brazil. 1,687 likes · 382 were here. Estacionamento próprio....</t>
+          <t>A empresa Barbearia Curitiba trabalha na categoria Barbearias na cidade de Ortigueira, PR na R. Ader...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://www.solutudo.com.br/empresas/pr/ortigueira/barbearias/barbearia-curitiba-22243010</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>(41) 99769-4378</t>
+          <t>(41) 3057-1357</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>5541997694378</t>
+          <t>554130571357</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20378%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20curitiba</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia 378 aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barbearia Curitiba em Ortigueira, PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1090,29 +1086,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia 378?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba em Ortigueira, PR?</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://wa.me/5541997694378?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20378%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554130571357?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>https://wa.me/5541997694378?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20378%3F</t>
+          <t>https://wa.me/554130571357?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%3F</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Barbearia Curitiba Oficial Cajuru PR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Porto - Barbearia - Água Verde - Curitiba</t>
+          <t>Barbearia Curitiba Oficial Cajuru PR - Telefone... | Bendito Guia</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1127,7 +1123,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Porto Barbearia · Formas de pagamento: ... TV, Aceita cartão de crédito · location_on · Rua Rua Brig...</t>
+          <t>Sobre a Empresa. Conheça a Barbearia Curitiba Oficial Cajuru PR, referência absoluta quando o assunt...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1137,28 +1133,24 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.trinks.com/porto</t>
+          <t>https://www.benditoguia.com.br/empresa/barbearia-curitiba-oficial-cajuru-pr</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>(41) 99979-3362</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>5541999793362</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Porto%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20curitiba</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Porto aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Curitiba Oficial Cajuru PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1168,29 +1160,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Porto?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Oficial Cajuru PR?</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://wa.me/5541999793362?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Porto%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>https://wa.me/5541999793362?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Porto%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%3F</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BARBER TOWN</t>
+          <t>Barbearia Saint Germain</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BARBER TOWN - BARBEARIA, Curitiba - Comentários de Restaurantes</t>
+          <t>Barbearia Saint Germain em Curitiba, PR | MestreGeo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1205,7 +1197,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Todos os restaurantes em CuritibaRestaurantes perto de Barber Town - BarbeariaCozinhas populares em ...</t>
+          <t>Informações completas da organização BARBEARIA SAINT GERMAIN LTDA em Curitiba, Paraná. CNPJ: 36.748....</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1215,24 +1207,28 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.tripadvisor.com.br/Restaurant_Review-g303441-d11180533-Reviews-Barber_Town_Barbearia-Curitiba_State_of_Parana.html</t>
+          <t>https://mestregeo.com.br/cnpj/pr/curitiba/barbearia-saint-germain-36748126000196</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>(CU) 98877-6655</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
+          <t>(41) 99894-4124</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>5541998944124</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/BARBER%20TOWN%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Saint%20Germain%20curitiba</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da BARBER TOWN aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Saint Germain aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1242,29 +1238,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a BARBER TOWN?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Saint Germain?</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20BARBER%20TOWN%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Saint%20Germain%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20BARBER%20TOWN%3F</t>
+          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Saint%20Germain%3F</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Centro</t>
+          <t>Barbearia perto de mim</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Centro | TikTok</t>
+          <t>Barbearia perto de mim em Curitiba - PR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1279,17 +1275,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Barbearia clássica no Centro de Curitiba. #barbearia #curitiba #barbeariaclassica.Conheça a Barbeari...</t>
+          <t>Aqui você encontra uma seleção completa das melhores Barbearia próximas da sua localização, com aval...</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SITE FORA DO AR / LINK QUEBRADO 🚨</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/discover/barbearia-curitiba-centro</t>
+          <t>https://www.locaisdobrasil.com.br/encontre/barbearia-perto-de-mim-em-curitiba-pr</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1300,13 +1296,13 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Centro%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20perto%20de%20mim%20curitiba</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba Centro aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
+Vi o perfil da Barbearia perto de mim aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1316,29 +1312,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Centro?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia perto de mim?</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20Centro%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20perto%20de%20mim%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20Centro%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20perto%20de%20mim%3F</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba</t>
+          <t>Os melhores barbeiros perto de mim</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba | Corte Masculino e Barba na Régua</t>
+          <t>Os melhores barbeiros perto de mim em Curitiba - Fresha</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1353,7 +1349,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Barbearia em Curitiba: corte masculino, degradê e barba na navalha. Ambiente premium, atendimento po...</t>
+          <t>Agendar online com os melhores Barbeiros perto de você em Curitiba. Excelentes ofertas e descontos! ...</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1363,7 +1359,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://barbeariacuritiba.online/</t>
+          <t>https://www.fresha.com/lp/pt/bt/barbearias/br-curitiba</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1374,13 +1370,13 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20curitiba</t>
+          <t>https://www.google.com/maps/search/Os%20melhores%20barbeiros%20perto%20de%20mim%20curitiba</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Os melhores barbeiros perto de mim aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1390,29 +1386,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Os melhores barbeiros perto de mim?</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Os%20melhores%20barbeiros%20perto%20de%20mim%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Os%20melhores%20barbeiros%20perto%20de%20mim%3F</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Melhores Servios de Barbearias</t>
+          <t>Link to facebook.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Melhores Serviços de Barbearias em Curitiba, PR | GuiaFix</t>
+          <t>Link to facebook.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1427,38 +1423,34 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Descubra a Soul Barbearia, localizada no Shopping Estação de Curitiba. Nossa barbearia oferece um am...</t>
+          <t>The site owner hides the web page description....</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://guiafix.com.br/curitiba-pr/barbearias</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>(41) 99894-4124</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>5541998944124</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Melhores%20Servios%20de%20Barbearias%20curitiba</t>
+          <t>https://www.google.com/maps/search/Link%20to%20facebook.com%20curitiba</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Melhores Servios de Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Link to facebook.com aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1468,29 +1460,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Melhores Servios de Barbearias?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Link to facebook.com?</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Melhores%20Servios%20de%20Barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Link%20to%20facebook.com%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Melhores%20Servios%20de%20Barbearias%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Link%20to%20facebook.com%3F</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Barbers In Barbearia</t>
+          <t>Link to instagram.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Barbers In Barbearia - Curitiba - Faça Agendamentos Online - Preç</t>
+          <t>Link to instagram.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1505,38 +1497,34 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Confira Barbers In Barbearia em Curitiba - explore preços, avaliações e faça agendamentos online 24 ...</t>
+          <t>The site owner hides the web page description....</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://booksy.com/pt-br/99716_barbers-in-barbearia_barbearias_583853_curitiba</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>(41) 3598-9540</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>554135989540</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbers%20In%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Link%20to%20instagram.com%20curitiba</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbers In Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Link to instagram.com aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1546,29 +1534,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbers In Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Link to instagram.com?</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>https://wa.me/554135989540?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbers%20In%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Link%20to%20instagram.com%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>https://wa.me/554135989540?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbers%20In%20Barbearia%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Link%20to%20instagram.com%3F</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>JR BARBEARIA CURITIBA</t>
+          <t>Barbearia Curitiba Centro</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>JR BARBEARIA CURITIBA | Linktree</t>
+          <t>Barbearia Curitiba Centro | TikTok</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1583,38 +1571,34 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>JR BARBEARIA CURITIBA. Seu estilo começa aqui!. NOSSO WhatsApp. Conta comercial. ESTACIONAMENTO PARA...</t>
+          <t>Barbearia clássica no Centro de Curitiba. #barbearia #curitiba #barbeariaclassica.Conheça a Barbeari...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
+          <t>SITE FORA DO AR / LINK QUEBRADO 🚨</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://www.tiktok.com/discover/barbearia-curitiba-centro</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>(62) 7903-3700</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>556279033700</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/JR%20BARBEARIA%20CURITIBA%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Centro%20curitiba</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da JR BARBEARIA CURITIBA aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Barbearia Curitiba Centro aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1624,29 +1608,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a JR BARBEARIA CURITIBA?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Centro?</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://wa.me/556279033700?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20JR%20BARBEARIA%20CURITIBA%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20Centro%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>https://wa.me/556279033700?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20JR%20BARBEARIA%20CURITIBA%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20Centro%3F</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba em Ortigueira, PR</t>
+          <t>Barbers In Barbearia</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba em Ortigueira, PR | Barbearias | Solutudo</t>
+          <t>Barbers In Barbearia - Curitiba - Faça Agendamentos Online - Preç</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1661,7 +1645,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A empresa Barbearia Curitiba trabalha na categoria Barbearias na cidade de Ortigueira, PR na R. Ader...</t>
+          <t>Confira Barbers In Barbearia em Curitiba - explore preços, avaliações e faça agendamentos online 24 ...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1671,28 +1655,28 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.solutudo.com.br/empresas/pr/ortigueira/barbearias/barbearia-curitiba-22243010</t>
+          <t>https://booksy.com/pt-br/99716_barbers-in-barbearia_barbearias_583853_curitiba</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>(41) 3057-1357</t>
+          <t>(41) 3598-9540</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>554130571357</t>
+          <t>554135989540</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbers%20In%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba em Ortigueira, PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbers In Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1702,29 +1686,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba em Ortigueira, PR?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbers In Barbearia?</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://wa.me/554130571357?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554135989540?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbers%20In%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>https://wa.me/554130571357?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20em%20Ortigueira%2C%20PR%3F</t>
+          <t>https://wa.me/554135989540?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbers%20In%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Oficial Cajuru PR</t>
+          <t>Barbearias / Barbeiros</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Barbearia Curitiba Oficial Cajuru PR - Telefone... | Bendito Guia</t>
+          <t>Barbearias / Barbeiros em Curitiba, PR — WhatsApp</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1739,17 +1723,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sobre a Empresa. Conheça a Barbearia Curitiba Oficial Cajuru PR, referência absoluta quando o assunt...</t>
+          <t>Barbeiro em Curitiba — Guia Completo para Escolher o Melhor Profissional. Contratar um barbeiro em C...</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.benditoguia.com.br/empresa/barbearia-curitiba-oficial-cajuru-pr</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1760,13 +1744,13 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearias%20/%20Barbeiros%20curitiba</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Curitiba Oficial Cajuru PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearias / Barbeiros aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1776,29 +1760,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba Oficial Cajuru PR?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearias / Barbeiros?</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearias%20/%20Barbeiros%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%20Oficial%20Cajuru%20PR%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearias%20/%20Barbeiros%3F</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Barbearia em Centro</t>
+          <t>Barbearia Curitiba</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Barbearia em Centro | Gustavinho do Corte - CIC Curitiba</t>
+          <t>Barbearia Curitiba | Corte Masculino e Barba na Régua</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1813,7 +1797,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Barbearia perto do Centro, a 10 km. Corte R$50, Barba R$50. Agende pelo WhatsApp....</t>
+          <t>Barbearia em Curitiba: corte masculino, degradê e barba na navalha. Ambiente premium, atendimento po...</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1823,7 +1807,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.barbeiro.curitiba.br/bairros/centro</t>
+          <t>https://barbeariacuritiba.online/</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1834,13 +1818,13 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20em%20Centro%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Curitiba%20curitiba</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia em Centro aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Curitiba aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1850,29 +1834,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia em Centro?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Curitiba?</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20em%20Centro%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20em%20Centro%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Curitiba%3F</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Don Barbearia</t>
+          <t>Melhores Servios de Barbearias</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Don Barbearia | Curitiba PR</t>
+          <t>Melhores Serviços de Barbearias em Curitiba, PR | GuiaFix</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1887,38 +1871,38 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Don Barbearia, Curitiba, Brazil. 625 likes · 228 were here. - BARBA - CABELO - BIGODE ***Atendimento...</t>
+          <t>Descubra a Soul Barbearia, localizada no Shopping Estação de Curitiba. Nossa barbearia oferece um am...</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://guiafix.com.br/curitiba-pr/barbearias</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>(41) 3501-0365</t>
+          <t>(41) 99894-4124</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>554135010365</t>
+          <t>5541998944124</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Don%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Melhores%20Servios%20de%20Barbearias%20curitiba</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Don Barbearia aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Melhores Servios de Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -1928,29 +1912,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Don Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Melhores Servios de Barbearias?</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://wa.me/554135010365?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Don%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Melhores%20Servios%20de%20Barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>https://wa.me/554135010365?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Don%20Barbearia%3F</t>
+          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Melhores%20Servios%20de%20Barbearias%3F</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Barbearias / Barbeiros</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Barbearias / Barbeiros em Curitiba, PR — WhatsApp</t>
+          <t>Sistema Agendamento Barbearia Curitiba: O Melhor em... | AgendZap</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1965,38 +1949,34 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Em Curitiba, a Barbearia Goldman é uma Barbearia voltada ao público masculino, com ambiente intimist...</t>
+          <t>Veja como ele vai mudar a sua barbearia: Agendamento Automático 24h pelo WhatsApp: Seus clientes age...</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SEM SITE (OPORTUNIDADE QUENTE 🔥)</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Sem Site Cadastrado</t>
+          <t>https://agendzap.com.br/blog/barbearia/barbershop-em-curitiba-melhor-sistema-de-agenda-2026-107</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>(41) 99894-4124</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>5541998944124</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearias%20/%20Barbeiros%20curitiba</t>
+          <t>https://www.google.com/maps/search/Sistema%20curitiba</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearias / Barbeiros aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
+Vi o perfil da Sistema aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2006,29 +1986,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearias / Barbeiros?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Sistema?</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998944124?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearias%20/%20Barbeiros%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Sistema%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998944124?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearias%20/%20Barbeiros%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Sistema%3F</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BARBEARIA DON VITO</t>
+          <t>Kontato para Barbearia</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BARBEARIA DON VITO - BARBEARIA CURITIBA (41) 99879-0994</t>
+          <t>Kontato para Barbearia em Curitiba PR — IA, agenda e cobrança no.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2043,38 +2023,34 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>June 26, 2023 - Barbearia Curitiba, Corte de cabelo masculino, Barba, Estilo masculino, Barbeiro, Ap...</t>
+          <t>Barbearia em Curitiba/PR — atendente IA, agenda online, cobrança Pix e fidelidade no WhatsApp. Clien...</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SITE FORA DO AR / LINK QUEBRADO 🚨</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://barbeariadonvito.curitiba.br/</t>
+          <t>https://kontato.themagicbox.app/site/segmento/barbearia/curitiba</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>(41) 99879-0994</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>5541998790994</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/BARBEARIA%20DON%20VITO%20curitiba</t>
+          <t>https://www.google.com/maps/search/Kontato%20para%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da BARBEARIA DON VITO aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
+Vi o perfil da Kontato para Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2084,29 +2060,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a BARBEARIA DON VITO?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Kontato para Barbearia?</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998790994?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20BARBEARIA%20DON%20VITO%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Kontato%20para%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998790994?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20BARBEARIA%20DON%20VITO%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Kontato%20para%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mon's Barbearia</t>
+          <t>Sistema para Barbearia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mon's Barbearia | Curitiba e Pinhais</t>
+          <t>Sistema para Barbearia em Curitiba — Agenda e WhatsApp 24h</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2121,7 +2097,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Na Mon's Barbearia, você é o centro das atenções. Barba, cabelo e bigode como você merece!Muito expe...</t>
+          <t>Sistema de gestão para barbearia em Curitiba (PR) com bot WhatsApp 24h, agenda por barbeiro, comissã...</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2131,28 +2107,24 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.monsbarbearia.com.br/</t>
+          <t>https://operosistemas.com.br/sistema-para-barbearia/curitiba</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>(41) 3226-3040</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>554132263040</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Mon%27s%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Sistema%20para%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Mon's Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Sistema para Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2162,29 +2134,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Mon's Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Sistema para Barbearia?</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>https://wa.me/554132263040?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Mon%27s%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Sistema%20para%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>https://wa.me/554132263040?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Mon%27s%20Barbearia%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Sistema%20para%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Channel's Centro de Beleza e Barbearia, Curit</t>
+          <t>Squad Barbearia Official: Instagram</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Channel's Centro de Beleza e Barbearia, Curitiba — R. Dom Pedro..</t>
+          <t>Squad Barbearia Official: Instagram | Linktree</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2199,38 +2171,34 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Para ter uma visão melhor da localização "Channel's Centro de Beleza e Barbearia", preste atenção na...</t>
+          <t>Squad Barbearia has been a member of Linktree for 6 years and joined in December 2019. The social me...</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://br.polomap.com/curitiba/8685</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>(41) 3243-8787</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>554132438787</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Channel%27s%20Centro%20de%20Beleza%20e%20Barbearia%2C%20Curit%20curitiba</t>
+          <t>https://www.google.com/maps/search/Squad%20Barbearia%20Official%3A%20Instagram%20curitiba</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Channel's Centro de Beleza e Barbearia, Curit aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Squad Barbearia Official: Instagram aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2240,29 +2208,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Channel's Centro de Beleza e Barbearia, Curit?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Squad Barbearia Official: Instagram?</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://wa.me/554132438787?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Channel%27s%20Centro%20de%20Beleza%20e%20Barbearia%2C%20Curit%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Squad%20Barbearia%20Official%3A%20Instagram%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>https://wa.me/554132438787?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Channel%27s%20Centro%20de%20Beleza%20e%20Barbearia%2C%20Curit%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Squad%20Barbearia%20Official%3A%20Instagram%3F</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Barbearia VIP</t>
+          <t>Barbearia Business Club</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Barbearia VIP — Barbearia Premium desde 1998</t>
+          <t>Barbearia Business Club - Bem-Vindo a BBC</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2277,7 +2245,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pioneiros em barbearia premium desde 1998. Mais de 40 unidades em seis estados do Brasil. Experiênci...</t>
+          <t>A Bussines Club tem como objetivo proporcionar ao homem uma extraordinária experiência em barbearia ...</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2287,24 +2255,28 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://barbeariavip.com.br/</t>
+          <t>https://www.barbeariabusinessclub.com.br/</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>(CU) 98877-6655</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>(41) 9870-0693</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>554198700693</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20VIP%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Business%20Club%20curitiba</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia VIP aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Business Club aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2314,29 +2286,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia VIP?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Business Club?</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20VIP%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554198700693?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Business%20Club%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20VIP%3F</t>
+          <t>https://wa.me/554198700693?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Business%20Club%3F</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Salo De Beleza E Barbearia Family Hair a Curi</t>
+          <t>316barbearia</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Salão De Beleza E Barbearia Family Hair a Curitiba - Infobel</t>
+          <t>316barbearia | Instagram | Linktree</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2351,38 +2323,34 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Salão De Beleza E Barbearia Family Hair 5.0 5.0(38 classificações) Rua Nossa Senhora de Nazaré 1641 ...</t>
+          <t>@316barbearia Avenida Senador Salgado Filho, 4761 ; Loja 5, Curitiba. APLICATIVO DE AGENDAMENTO ONLI...</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SITE ATIVO 📱</t>
+          <t>SEM SITE PRÓPRIO (OPORTUNIDADE 🔥)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.infobel.com/pt/brazil/salao_de_beleza_e_barbearia_family_hair/curitiba/BR156193478-4130395072/businessdetails.aspx</t>
+          <t>Sem Site Cadastrado</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>(41) 3039-5072</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>554130395072</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%20curitiba</t>
+          <t>https://www.google.com/maps/search/316barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Salo De Beleza E Barbearia Family Hair a Curi aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da 316barbearia aí em Curitiba no Google e vi que vocês ainda não têm um site próprio para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2392,29 +2360,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Salo De Beleza E Barbearia Family Hair a Curi?</t>
+Posso te mandar a prévia demonstrativa que fiz para a 316barbearia?</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>https://wa.me/554130395072?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20316barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20voc%C3%AAs%20ainda%20n%C3%A3o%20t%C3%AAm%20um%20site%20pr%C3%B3prio%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>https://wa.me/554130395072?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20316barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Melhores sales de beleza</t>
+          <t>Mon's Barbearia</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Melhores salões de beleza em Curitiba - FreshaBarbearia Clube | T</t>
+          <t>Mon's Barbearia | Curitiba e Pinhais</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2429,7 +2397,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Agendar online com os melhores salões em Curitiba. Excelentes ofertas e descontos! Ver avaliações e ...</t>
+          <t>Na Mon's Barbearia, você é o centro das atenções. Barba, cabelo e bigode como você merece!Muito expe...</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2439,24 +2407,28 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.fresha.com/lp/pt/br-curitiba</t>
+          <t>https://www.monsbarbearia.com.br/</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>(CU) 98877-6655</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
+          <t>(52) 0484-2600</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>555204842600</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Melhores%20sales%20de%20beleza%20curitiba</t>
+          <t>https://www.google.com/maps/search/Mon%27s%20Barbearia%20curitiba</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Melhores sales de beleza aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Mon's Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2466,29 +2438,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Melhores sales de beleza?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Mon's Barbearia?</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Melhores%20sales%20de%20beleza%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/555204842600?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Mon%27s%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Melhores%20sales%20de%20beleza%3F</t>
+          <t>https://wa.me/555204842600?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Mon%27s%20Barbearia%3F</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sales de Beleza</t>
+          <t>Don Barbearia, Curitiba</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Salões de Beleza em Curitiba | Expert Beauty Center</t>
+          <t>Don Barbearia, Curitiba — R. Vieira dos Santos, telefone...</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2503,7 +2475,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>O Expert Beauty Center é a maior e mais completa rede de salões de Curitiba. Com unidades nos endere...</t>
+          <t>Don Barbearia. Fechado. Curitiba, R. Vieira dos Santos, 162.(751 metro), Barbearia 1 (820 m), Barbea...</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2513,24 +2485,28 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.expertbeautycenter.com.br/</t>
+          <t>https://br.polomap.com/curitiba/8735</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>(CU) 98877-6655</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+          <t>(41) 3501-0365</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>554135010365</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Sales%20de%20Beleza%20curitiba</t>
+          <t>https://www.google.com/maps/search/Don%20Barbearia%2C%20Curitiba%20curitiba</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Sales de Beleza aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Don Barbearia, Curitiba aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2540,29 +2516,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Sales de Beleza?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Don Barbearia, Curitiba?</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Sales%20de%20Beleza%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554135010365?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Don%20Barbearia%2C%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Sales%20de%20Beleza%3F</t>
+          <t>https://wa.me/554135010365?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Don%20Barbearia%2C%20Curitiba%3F</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Barber Club</t>
+          <t>A BANCA CURITIBA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Barber Club - Barbearia Centro Curitiba PR - Telefone, Endereço e</t>
+          <t>A BANCA CURITIBA | CNPJ 53.441.822/0001-74 | GuiaPJ</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2577,7 +2553,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Barber Club - Barbearia Centro Curitiba PR fica na R. Saldanha Marinho, 1267 - Centro, Curitiba - PR...</t>
+          <t>A empresa BARBEARIA CURITIBA LTDA, CNPJ 53.441.822/0001-74, iniciou suas atividades em 10/01/2024. A...</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2587,28 +2563,24 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.benditoguia.com.br/empresa/barber-club-barbearia-centro-curitiba-pr</t>
+          <t>https://guiapj.com.br/consulta-cnpj/53441822000174</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>(41) 99866-9546</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>5541998669546</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barber%20Club%20curitiba</t>
+          <t>https://www.google.com/maps/search/A%20BANCA%20CURITIBA%20curitiba</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barber Club aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da A BANCA CURITIBA aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2618,29 +2590,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barber Club?</t>
+Posso te mandar a prévia demonstrativa que fiz para a A BANCA CURITIBA?</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998669546?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barber%20Club%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20A%20BANCA%20CURITIBA%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>https://wa.me/5541998669546?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barber%20Club%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20A%20BANCA%20CURITIBA%3F</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Barbearia Rodrigues</t>
+          <t>Salo De Beleza E Barbearia Family Hair a Curi</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Barbearia Rodrigues: telefone y horário - Rua Curitiba 778 Sala 1</t>
+          <t>Salão De Beleza E Barbearia Family Hair a Curitiba - Infobel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2655,7 +2627,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Barbearias, wellness, distrito - Dirección: Rua Curitiba 778 Sala 103 - Belo Horizonte, Minas Gerais...</t>
+          <t>Salão De Beleza E Barbearia Family Hair 5.0 5.0(38 classificações) Rua Nossa Senhora de Nazaré 1641 ...</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2665,28 +2637,28 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.planetabrasileiro.com/barbearia-rodrigues-F1009C80E1AD043</t>
+          <t>https://www.infobel.com/pt/brazil/salao_de_beleza_e_barbearia_family_hair/curitiba/BR156193478-4130395072/businessdetails.aspx</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>(03) 1989-6889</t>
+          <t>(41) 3039-5072</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>550319896889</t>
+          <t>554130395072</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Rodrigues%20curitiba</t>
+          <t>https://www.google.com/maps/search/Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%20curitiba</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Rodrigues aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Salo De Beleza E Barbearia Family Hair a Curi aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2696,29 +2668,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Rodrigues?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Salo De Beleza E Barbearia Family Hair a Curi?</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>https://wa.me/550319896889?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Rodrigues%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554130395072?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>https://wa.me/550319896889?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Rodrigues%3F</t>
+          <t>https://wa.me/554130395072?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Salo%20De%20Beleza%20E%20Barbearia%20Family%20Hair%20a%20Curi%3F</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Barbearia Moustache</t>
+          <t>Barbearia VIP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Barbearia Moustache - Cabral 31151716000113 Curitiba</t>
+          <t>Barbearia VIP — Barbearia Premium desde 1998</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2733,7 +2705,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>O telefone da empresa é (41) 3669-**** essa informação podem ser vistas na sessão contato dessa pagi...</t>
+          <t>Pioneiros em barbearia premium desde 1998. Mais de 40 unidades em seis estados do Brasil. Experiênci...</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2743,28 +2715,24 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://cnpj.biz/31151716000113</t>
+          <t>https://barbeariavip.com.br/</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>(31) 1517-1600</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>553115171600</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Moustache%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20VIP%20curitiba</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Moustache aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia VIP aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2774,29 +2742,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Moustache?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia VIP?</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>https://wa.me/553115171600?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Moustache%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20VIP%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>https://wa.me/553115171600?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Moustache%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20VIP%3F</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Baro da Navalha</t>
+          <t>Sales de Beleza</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Barão da Navalha | Barbearia Curitiba Centro Cívico</t>
+          <t>Salões de Beleza em Curitiba | Expert Beauty Center</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2811,7 +2779,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Chegamos Curitiba! A Barão chega na cidade mais charmosa do Brasil com um conceito diferenciado de b...</t>
+          <t>O Expert Beauty Center é a maior e mais completa rede de salões de Curitiba. Com unidades nos endere...</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2821,28 +2789,24 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://baraodanavalha.com.br/barbearia-curitiba-centro-civico/</t>
+          <t>https://www.expertbeautycenter.com.br/</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>(41) 3085-8475</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>554130858475</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Baro%20da%20Navalha%20curitiba</t>
+          <t>https://www.google.com/maps/search/Sales%20de%20Beleza%20curitiba</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Baro da Navalha aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Sales de Beleza aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2852,29 +2816,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Baro da Navalha?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Sales de Beleza?</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>https://wa.me/554130858475?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Baro%20da%20Navalha%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Sales%20de%20Beleza%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>https://wa.me/554130858475?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Baro%20da%20Navalha%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Sales%20de%20Beleza%3F</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Barbearia Original</t>
+          <t>Salo de beleza Studio NB Curitiba Batel PR</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Barbearia Original em Curitiba-PR - Barbearias Perto de Mim</t>
+          <t>Salão de beleza Studio NB Curitiba Batel PR - Telefone ...</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2889,7 +2853,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>October 19, 2020 - A loja física está localizada no bairro Hauer, em Curitiba - PR. A data de abertu...</t>
+          <t>Procurando por Salão de beleza Studio NB Curitiba Batel PR? Aqui você encontra contato completo, hor...</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2899,28 +2863,24 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://barbeariaspertodemim.com/e/barbearia-original-aphqje/</t>
+          <t>https://www.benditoguia.com.br/empresa/salao-de-beleza-studio-nb-curitiba-batel-pr</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>(17) 3939-9700</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>551739399700</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Original%20curitiba</t>
+          <t>https://www.google.com/maps/search/Salo%20de%20beleza%20Studio%20NB%20Curitiba%20Batel%20PR%20curitiba</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Original aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Salo de beleza Studio NB Curitiba Batel PR aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -2930,29 +2890,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Original?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Salo de beleza Studio NB Curitiba Batel PR?</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>https://wa.me/551739399700?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Original%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Salo%20de%20beleza%20Studio%20NB%20Curitiba%20Batel%20PR%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>https://wa.me/551739399700?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Original%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Salo%20de%20beleza%20Studio%20NB%20Curitiba%20Batel%20PR%3F</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Barbearia Seu Julio</t>
+          <t>MEN’S</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Barbearia Seu Julio | Barbearia em Curitiba, Barbearia no Novo...</t>
+          <t>MEN’S — Clínica de Estética Masculina</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2967,7 +2927,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>A Tradicional Barbearia. A Barbearia Seu Júlio nasceu da paixão pela tradição e pelo estilo. Nossa m...</t>
+          <t>Estética premium para homens: barbearia, depilação a laser, harmonização, transplante capilar, masso...</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2977,28 +2937,28 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://barbeariaseujulio.com.br/</t>
+          <t>https://www.mensoficial.com.br/</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>(41) 3039-5411</t>
+          <t>(15) 6695-4376</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>554130395411</t>
+          <t>551566954376</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20Seu%20Julio%20curitiba</t>
+          <t>https://www.google.com/maps/search/MEN%E2%80%99S%20curitiba</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia Seu Julio aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da MEN’S aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3008,29 +2968,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia Seu Julio?</t>
+Posso te mandar a prévia demonstrativa que fiz para a MEN’S?</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>https://wa.me/554130395411?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Seu%20Julio%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/551566954376?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20MEN%E2%80%99S%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>https://wa.me/554130395411?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Seu%20Julio%3F</t>
+          <t>https://wa.me/551566954376?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20MEN%E2%80%99S%3F</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Shelby Barbearia</t>
+          <t>Barbearia Seu Julio</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Shelby Barbearia - (41) 98475-3472 BARBEARIA EM CURITIBA...</t>
+          <t>Barbearia Seu Julio | Barbearia em Curitiba, Barbearia no Novo...</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3045,7 +3005,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Na Shelby Barbearia, o atendimento é personalizado e pensado para realçar o melhor de cada cliente, ...</t>
+          <t>A Tradicional Barbearia. A Barbearia Seu Júlio nasceu da paixão pela tradição e pelo estilo. Nossa m...</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3055,28 +3015,28 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://barbeariashelby.com.br/spa-da-barba/</t>
+          <t>https://barbeariaseujulio.com.br/</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>(41) 98475-3472</t>
+          <t>(41) 3039-5411</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>5541984753472</t>
+          <t>554130395411</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Shelby%20Barbearia%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Seu%20Julio%20curitiba</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Shelby Barbearia aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Seu Julio aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3086,29 +3046,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Shelby Barbearia?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Seu Julio?</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>https://wa.me/5541984753472?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Shelby%20Barbearia%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554130395411?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Seu%20Julio%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>https://wa.me/5541984753472?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Shelby%20Barbearia%3F</t>
+          <t>https://wa.me/554130395411?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Seu%20Julio%3F</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>147 avaliaes sobre Unik Barbearia (Barbearia)</t>
+          <t>Barbearia Goldman</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>147 avaliações sobre Unik Barbearia (Barbearia) em Curitiba (Para</t>
+          <t>Barbearia Goldman</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3123,7 +3083,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Avaliações » Barbearia » Paraná » Curitiba » Unik barbearia.Melhor barbearia de curitiba e região, a...</t>
+          <t>Barbearia Goldman. Barbearia Goldman A Melhor de Curitiba. Sinta essa Experiência....</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3133,28 +3093,28 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://avaliacoesbrasil.com/barbearia/curitiba/unik-barbearia/</t>
+          <t>https://www.barbeariagoldman.com.br/</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>(99) 8510-5843</t>
+          <t>(41) 99702-3434</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>559985105843</t>
+          <t>5541997023434</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/147%20avaliaes%20sobre%20Unik%20Barbearia%20%28Barbearia%29%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20Goldman%20curitiba</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da 147 avaliaes sobre Unik Barbearia (Barbearia) aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Barbearia Goldman aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3164,29 +3124,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a 147 avaliaes sobre Unik Barbearia (Barbearia)?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia Goldman?</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>https://wa.me/559985105843?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20147%20avaliaes%20sobre%20Unik%20Barbearia%20%28Barbearia%29%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541997023434?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20Goldman%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>https://wa.me/559985105843?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20147%20avaliaes%20sobre%20Unik%20Barbearia%20%28Barbearia%29%3F</t>
+          <t>https://wa.me/5541997023434?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20Goldman%3F</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Overall Barber</t>
+          <t>10 melhores barbeiros para Curitiba</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Overall Barber - (41) 98488-0758 Barbearia em Curitiba BARBEARIA.</t>
+          <t>10 melhores barbeiros para Curitiba</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3201,7 +3161,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Seu clube vai além da barbearia. Tenha acesso a descontos exclusivos nos parceiros: 02.Contato. R. J...</t>
+          <t>80020-340 Curitiba. Atentendo na barbearia Johnny Navalha, além disso domingo e segunda, disponivel ...</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3211,28 +3171,24 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://barbeariaoverall.com.br/planos/</t>
+          <t>https://www.starofservice.com.br/dir/parana/curitiba/curitiba/servico-de-barbearia</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>(41) 98488-0758</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>5541984880758</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Overall%20Barber%20curitiba</t>
+          <t>https://www.google.com/maps/search/10%20melhores%20barbeiros%20para%20Curitiba%20curitiba</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Overall Barber aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da 10 melhores barbeiros para Curitiba aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3242,29 +3198,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Overall Barber?</t>
+Posso te mandar a prévia demonstrativa que fiz para a 10 melhores barbeiros para Curitiba?</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>https://wa.me/5541984880758?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Overall%20Barber%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%2010%20melhores%20barbeiros%20para%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>https://wa.me/5541984880758?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Overall%20Barber%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%2010%20melhores%20barbeiros%20para%20Curitiba%3F</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Mercado de Barbearia em Centro, Curitiba 2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Sistema Agendamento Barbearia Curitiba: O Melhor em... | AgendZap</t>
+          <t>Mercado de Barbearia em Centro, Curitiba 2026 | OndeAbrir</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3279,7 +3235,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ter um atendimento rápido e eficiente, sem filas de espera ou mensagens perdidas. Focar no que realm...</t>
+          <t>Mercado de barbearias em Centro, Curitiba: como está em 2026? Cenário competitivo de barbearias em C...</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3289,7 +3245,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://agendzap.com.br/blog/barbearia/barbershop-em-curitiba-melhor-sistema-de-agenda-2026-107</t>
+          <t>https://ondeabrir.com/mercado/barbearia/curitiba/centro</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3300,13 +3256,13 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Sistema%20curitiba</t>
+          <t>https://www.google.com/maps/search/Mercado%20de%20Barbearia%20em%20Centro%2C%20Curitiba%202026%20curitiba</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Sistema aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
+Vi o perfil da Mercado de Barbearia em Centro, Curitiba 2026 aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3316,29 +3272,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Sistema?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Mercado de Barbearia em Centro, Curitiba 2026?</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Sistema%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Mercado%20de%20Barbearia%20em%20Centro%2C%20Curitiba%202026%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Sistema%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Mercado%20de%20Barbearia%20em%20Centro%2C%20Curitiba%202026%3F</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Barbearia no Centro de Curitiba</t>
+          <t>Barbearia John Six</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Barbearia no Centro de Curitiba – Barba n Beer – Cabelereiro Masc</t>
+          <t>Barbearia John Six - Bigorrilho em Curitiba - PR | Locais do Bras</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3353,34 +3309,38 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Mas, se preferir, também trabalhamos com horários marcados que podem ser agendados por telefone ou w...</t>
+          <t>Barbearia John Six - Bigorrilho atua no ramo de Barbearia, horário de funcionamento quarta a quinta-...</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>SITE FORA DO AR / LINK QUEBRADO 🚨</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.barbanbeer.com.br/</t>
+          <t>https://www.locaisdobrasil.com.br/encontre/barbearia/curitiba-pr/barbearia-john-six-bigorrilho/61cf4338c76c53fe0914d004</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>(CU) 98877-6655</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
+          <t>(41) 1111-1111</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>554111111111</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barbearia%20no%20Centro%20de%20Curitiba%20curitiba</t>
+          <t>https://www.google.com/maps/search/Barbearia%20John%20Six%20curitiba</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barbearia no Centro de Curitiba aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
+Vi o perfil da Barbearia John Six aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3390,29 +3350,29 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barbearia no Centro de Curitiba?</t>
+Posso te mandar a prévia demonstrativa que fiz para a Barbearia John Six?</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20no%20Centro%20de%20Curitiba%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/554111111111?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barbearia%20John%20Six%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20no%20Centro%20de%20Curitiba%3F</t>
+          <t>https://wa.me/554111111111?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barbearia%20John%20Six%3F</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Barigui</t>
+          <t>AutoRank para Barbearias</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Barigui - La Mafia Barbearia</t>
+          <t>AutoRank para Barbearias em Curitiba | Seu Negócio na Primeira...</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3427,38 +3387,34 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>April 9, 2025 - a la mafia Curitiba – Barigui Inaugurada em 06 de setembro de 2024, a unidade BARIGU...</t>
+          <t>Barbearias em Curitiba. Coloque sua barbearia na primeira página do Google e atraia clientes buscand...</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>SITE FORA DO AR (ERRO 404) 🚨</t>
+          <t>SITE ATIVO 📱</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.lamafiabarbearia.com.br/unidades/barigui/</t>
+          <t>https://www.autorank.com.br/barbearia/curitiba</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>(41) 3514-5154</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>554135145154</t>
-        </is>
-      </c>
+          <t>(CU) 98877-6655</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/Barigui%20curitiba</t>
+          <t>https://www.google.com/maps/search/AutoRank%20para%20Barbearias%20curitiba</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
           <t>Olá, tudo bem? Meu nome é João, sou da agência Webfy. 🚀
-Vi o perfil da Barigui aí em Curitiba no Google e fui tentar acessar o site de vocês e vi que está fora do ar.
+Vi o perfil da AutoRank para Barbearias aí em Curitiba no Google e vi que o site de vocês está um pouco desatualizado para celular.
 Nós estamos selecionando 5 empresas na região para **GANHAR A CRIAÇÃO DE UM SITE NOVO 100% GRATUITO** para o nosso portfólio deste mês.
 Já deixei uma demonstração pronta. Posso te mandar o link para você dar uma olhada sem compromisso?</t>
         </is>
@@ -3468,17 +3424,17 @@
           <t>Show! Como te falei, a **criação e o desenvolvimento do site saem 100% GRATUITOS** (você economiza cerca de R$ 2.000 que é o valor de mercado). 🎁
 A única coisa necessária é a taxa anual de hospedagem e servidor (R$ 599/ano ou parcelado), que é a taxa padrão que todo site na internet precisa ter para ficar online no seu nome com domínio próprio (.com.br).
 Incluso: Hospedagem rápida para celular, suporte, botão de WhatsApp e presença no Google!
-Posso te mandar a prévia demonstrativa que fiz para a Barigui?</t>
+Posso te mandar a prévia demonstrativa que fiz para a AutoRank para Barbearias?</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>https://wa.me/554135145154?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20Barigui%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20fui%20tentar%20acessar%20o%20site%20de%20voc%C3%AAs%20e%20vi%20que%20est%C3%A1%20fora%20do%20ar.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
+          <t>https://wa.me/5541988776655?text=Ol%C3%A1%2C%20tudo%20bem%3F%20Meu%20nome%20%C3%A9%20Jo%C3%A3o%2C%20sou%20da%20ag%C3%AAncia%20Webfy.%20%F0%9F%9A%80%0A%0AVi%20o%20perfil%20da%20AutoRank%20para%20Barbearias%20a%C3%AD%20em%20Curitiba%20no%20Google%20e%20vi%20que%20o%20site%20de%20voc%C3%AAs%20est%C3%A1%20um%20pouco%20desatualizado%20para%20celular.%0A%0AN%C3%B3s%20estamos%20selecionando%205%20empresas%20na%20regi%C3%A3o%20para%20%2A%2AGANHAR%20A%20CRIA%C3%87%C3%83O%20DE%20UM%20SITE%20NOVO%20100%25%20GRATUITO%2A%2A%20para%20o%20nosso%20portf%C3%B3lio%20deste%20m%C3%AAs.%0A%0AJ%C3%A1%20deixei%20uma%20demonstra%C3%A7%C3%A3o%20pronta.%20Posso%20te%20mandar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20sem%20compromisso%3F</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>https://wa.me/554135145154?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20Barigui%3F</t>
+          <t>https://wa.me/5541988776655?text=Show%21%20Como%20te%20falei%2C%20a%20%2A%2Acria%C3%A7%C3%A3o%20e%20o%20desenvolvimento%20do%20site%20saem%20100%25%20GRATUITOS%2A%2A%20%28voc%C3%AA%20economiza%20cerca%20de%20R%24%202.000%20que%20%C3%A9%20o%20valor%20de%20mercado%29.%20%F0%9F%8E%81%0A%0AA%20%C3%BAnica%20coisa%20necess%C3%A1ria%20%C3%A9%20a%20taxa%20anual%20de%20hospedagem%20e%20servidor%20%28R%24%20599/ano%20ou%20parcelado%29%2C%20que%20%C3%A9%20a%20taxa%20padr%C3%A3o%20que%20todo%20site%20na%20internet%20precisa%20ter%20para%20ficar%20online%20no%20seu%20nome%20com%20dom%C3%ADnio%20pr%C3%B3prio%20%28.com.br%29.%0A%0AIncluso%3A%20Hospedagem%20r%C3%A1pida%20para%20celular%2C%20suporte%2C%20bot%C3%A3o%20de%20WhatsApp%20e%20presen%C3%A7a%20no%20Google%21%0A%0APosso%20te%20mandar%20a%20pr%C3%A9via%20demonstrativa%20que%20fiz%20para%20a%20AutoRank%20para%20Barbearias%3F</t>
         </is>
       </c>
     </row>

</xml_diff>